<commit_message>
Corrected Book02 Chapter 01-02
</commit_message>
<xml_diff>
--- a/content-pipeline/inputs/book02/b02_ch01_final.xlsx
+++ b/content-pipeline/inputs/book02/b02_ch01_final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://transre-my.sharepoint.com/personal/fau_transre_com/Documents/_OneDrive/_Operational_Tools/Github/GCSEChinese/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://transre-my.sharepoint.com/personal/fau_transre_com/Documents/_OneDrive/_Operational_Tools/Github/GCSEChinese/Inputs/Primary/二上/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_D7BA18347A1BA7369A92CCFF16D49442D3664B3D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{436B84AF-616D-4563-A2A0-3F275FEFA40A}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_D7BA18347A1BA7369A92CCFF16D49442D3664B3D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60E89F5C-CB77-4FE6-B3A7-D3BAEC38E50B}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1905" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57600" yWindow="-16350" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta" sheetId="1" r:id="rId1"/>
@@ -139,140 +139,140 @@
     <t>English</t>
   </si>
   <si>
-    <t>二上：揑彩泥（第六頁）
-今天的視藝課開始了，王老師對大家說：「今天，我們來舉辦一個『動物聚會』。請大家拿出彩泥，捏出你最喜歡的小動物吧！」說完，玉老師給我們做了示範，三下兩下就揑出了一隻可愛的小兔子。
-「我要揑一隻小青蛙。」我早已經手癢癢了。首先，我拿出一塊綠色彩泥，把它搓揉成橢圓形，小青蛙的身體做好了。然後，我揑了四條腿黏在小青蛙的身體上。接着，我用黑色彩泥揑了兩個小圓球做眼睛。最後，我把白色彩泥搓成許多小細條，黏到青蛙的背上。這樣，一隻可愛的小青蛙就活靈活現地出現在我面前了。我想：一隻小青蛙太孤單了。於是，我又用黑色彩泥搓成黑色的小球，揑出細細的尾巴，一隻小蝌蚪就做成了。
+    <t>Kneading playdough</t>
+  </si>
+  <si>
+    <t>視藝課</t>
+  </si>
+  <si>
+    <t>Visual Arts class</t>
+  </si>
+  <si>
+    <t>動物聚會</t>
+  </si>
+  <si>
+    <t>Animal gathering</t>
+  </si>
+  <si>
+    <t>示範</t>
+  </si>
+  <si>
+    <t>Demonstration</t>
+  </si>
+  <si>
+    <t>首先</t>
+  </si>
+  <si>
+    <t>Firstly</t>
+  </si>
+  <si>
+    <t>黏</t>
+  </si>
+  <si>
+    <t>Sticky / To stick</t>
+  </si>
+  <si>
+    <t>孤單</t>
+  </si>
+  <si>
+    <t>Lonely / Alone</t>
+  </si>
+  <si>
+    <t>相繼</t>
+  </si>
+  <si>
+    <t>One after another / Successively</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>BookID</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>ChapterID</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>ChapterTitle</t>
+  </si>
+  <si>
+    <t>Book 02 · Chapter 01: 揑彩泥</t>
+  </si>
+  <si>
+    <t>REVIEW: check Pinyin (fix multi-pronunciation errors) and ContextSentence (fix if wrong or missing).</t>
+  </si>
+  <si>
+    <t>Traditional</t>
+  </si>
+  <si>
+    <t>Pinyin (auto - review!)</t>
+  </si>
+  <si>
+    <t>ContextSentence (auto - review!)</t>
+  </si>
+  <si>
+    <t>niē cǎi ní</t>
+  </si>
+  <si>
+    <t>shì yì kè</t>
+  </si>
+  <si>
+    <t>dòng wù jù huì</t>
+  </si>
+  <si>
+    <t>shì fàn</t>
+  </si>
+  <si>
+    <t>shǒu xiān</t>
+  </si>
+  <si>
+    <t>首先，我拿出一塊綠色彩泥，把它搓揉成橢圓形，小青蛙的身體做好了。</t>
+  </si>
+  <si>
+    <t>nián</t>
+  </si>
+  <si>
+    <t>gū dān</t>
+  </si>
+  <si>
+    <t>我想：一隻小青蛙太孤單了。</t>
+  </si>
+  <si>
+    <t>xiāng jì</t>
+  </si>
+  <si>
+    <t>一隻隻可愛的小動物相繼在同學們的手中誕生，有小猴子、大象、老虎。</t>
+  </si>
+  <si>
+    <t>今天的視藝課開始了，王老師對大家說：「今天，我們來舉辦一個『動物聚會』。</t>
+  </si>
+  <si>
+    <t>二上：捏彩泥（第六頁）
+今天的視藝課開始了，王老師對大家說：「今天，我們來舉辦一個『動物聚會』。請大家拿出彩泥，捏出你最喜歡的小動物吧！」說完，玉老師給我們做了示範，三下兩下就捏出了一隻可愛的小兔子。
+「我要捏一隻小青蛙。」我早已經手癢癢了。首先，我拿出一塊綠色彩泥，把它搓揉成橢圓形，小青蛙的身體做好了。然後，我捏了四條腿黏在小青蛙的身體上。接着，我用黑色彩泥捏了兩個小圓球做眼睛。最後，我把白色彩泥搓成許多小細條，黏到青蛙的背上。這樣，一隻可愛的小青蛙就活靈活現地出現在我面前了。我想：一隻小青蛙太孤單了。於是，我又用黑色彩泥搓成黑色的小球，捏出細細的尾巴，一隻小蝌蚪就做成了。
 「成功了！」我高興地喊道。「我也做好了。」我朝旁邊一看，志文正得意洋洋地拿着一隻「小豬」。看它一隻眼睛大一隻眼睛小，我不禁「撲哧」笑出了聲。
 一隻隻可愛的小動物相繼在同學們的手中誕生，有小猴子、大象、老虎。。。還真是一次「動物聚會」呀。捏彩泥真有趣！</t>
   </si>
   <si>
-    <t>揑彩泥</t>
-  </si>
-  <si>
-    <t>Kneading playdough</t>
-  </si>
-  <si>
-    <t>視藝課</t>
-  </si>
-  <si>
-    <t>Visual Arts class</t>
-  </si>
-  <si>
-    <t>動物聚會</t>
-  </si>
-  <si>
-    <t>Animal gathering</t>
-  </si>
-  <si>
-    <t>示範</t>
-  </si>
-  <si>
-    <t>Demonstration</t>
-  </si>
-  <si>
-    <t>首先</t>
-  </si>
-  <si>
-    <t>Firstly</t>
-  </si>
-  <si>
-    <t>黏</t>
-  </si>
-  <si>
-    <t>Sticky / To stick</t>
-  </si>
-  <si>
-    <t>孤單</t>
-  </si>
-  <si>
-    <t>Lonely / Alone</t>
-  </si>
-  <si>
-    <t>相繼</t>
-  </si>
-  <si>
-    <t>One after another / Successively</t>
-  </si>
-  <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>BookID</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>ChapterID</t>
-  </si>
-  <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>ChapterTitle</t>
-  </si>
-  <si>
-    <t>Book 02 · Chapter 01: 揑彩泥</t>
-  </si>
-  <si>
-    <t>REVIEW: check Pinyin (fix multi-pronunciation errors) and ContextSentence (fix if wrong or missing).</t>
-  </si>
-  <si>
-    <t>Traditional</t>
-  </si>
-  <si>
-    <t>Pinyin (auto - review!)</t>
-  </si>
-  <si>
-    <t>ContextSentence (auto - review!)</t>
-  </si>
-  <si>
-    <t>niē cǎi ní</t>
-  </si>
-  <si>
-    <t>shì yì kè</t>
-  </si>
-  <si>
-    <t>dòng wù jù huì</t>
-  </si>
-  <si>
-    <t>shì fàn</t>
-  </si>
-  <si>
-    <t>shǒu xiān</t>
-  </si>
-  <si>
-    <t>首先，我拿出一塊綠色彩泥，把它搓揉成橢圓形，小青蛙的身體做好了。</t>
-  </si>
-  <si>
-    <t>nián</t>
-  </si>
-  <si>
-    <t>然後，我揑了四條腿黏在小青蛙的身體上。</t>
-  </si>
-  <si>
-    <t>gū dān</t>
-  </si>
-  <si>
-    <t>我想：一隻小青蛙太孤單了。</t>
-  </si>
-  <si>
-    <t>xiāng jì</t>
-  </si>
-  <si>
-    <t>一隻隻可愛的小動物相繼在同學們的手中誕生，有小猴子、大象、老虎。</t>
-  </si>
-  <si>
-    <t>今天的視藝課開始了，王老師對大家說：「今天，我們來舉辦一個『動物聚會』。</t>
-  </si>
-  <si>
-    <t>玉老師給我們做了示範，三下兩下就揑出了一隻可愛的小兔子。</t>
-  </si>
-  <si>
-    <t>二上：揑彩泥（第六頁）</t>
+    <t>捏彩泥</t>
+  </si>
+  <si>
+    <t>二上：捏彩泥（第六頁）</t>
+  </si>
+  <si>
+    <t>玉老師給我們做了示範，三下兩下就捏出了一隻可愛的小兔子。</t>
+  </si>
+  <si>
+    <t>然後，我捏了四條腿黏在小青蛙的身體上。</t>
   </si>
 </sst>
 </file>
@@ -299,18 +299,21 @@
       <sz val="14"/>
       <color rgb="FF2B6CB0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -661,87 +664,87 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" s="2"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" s="2"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" s="2"/>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" s="2"/>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B15" s="2"/>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B16" s="2"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B17" s="2"/>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B19" s="2"/>
     </row>
   </sheetData>
@@ -753,14 +756,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="80" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -771,198 +774,198 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3"/>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" s="3"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" s="3"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" s="3"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" s="3"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" s="3"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" s="3"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" s="3"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" s="3"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" s="3"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" s="3"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" s="3"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" s="3"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" s="3"/>
     </row>
   </sheetData>
@@ -974,154 +977,154 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="80.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="80.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
         <v>32</v>
       </c>
-      <c r="D4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
         <v>33</v>
-      </c>
-      <c r="D5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
       </c>
       <c r="D7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>13</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>36</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D10" t="s">
         <v>38</v>
       </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D11" t="s">
         <v>40</v>
-      </c>
-      <c r="D10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>